<commit_message>
Aplikacja dostępna na platformie Azure
</commit_message>
<xml_diff>
--- a/DigitalWars.Server/Initializers/DigitalWars_UserInitialization.xlsx
+++ b/DigitalWars.Server/Initializers/DigitalWars_UserInitialization.xlsx
@@ -604,7 +604,7 @@
     <t>Próbujesz udoskonalać proces jednak bariery wewnętrzne skutecznie to blokują. Pomyśl nad analizą danych czy zwiększeniem świadomości zespołu.</t>
   </si>
   <si>
-    <t>Cards_Weights_Id</t>
+    <t>CardsWeights_Id</t>
   </si>
   <si>
     <t>Weights_X</t>
@@ -12942,7 +12942,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="12.75" customHeight="1">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>190</v>
       </c>
       <c r="B1" s="10" t="s">

</xml_diff>